<commit_message>
Add unit to tick interval designation
So now you can specify 1y for 1 year ticks, 6m for 6m ticks, 30d for 30 day, etc.
</commit_message>
<xml_diff>
--- a/data/StoryDataExample.xlsx
+++ b/data/StoryDataExample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daschre\Documents\Projects\IRIS\scrolly-story-generator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB121AD1-1D26-47EA-8501-64B9F980BBB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EEDA41C-F330-4C4C-8496-518467B9A0A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51345" yWindow="-6195" windowWidth="38700" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-42255" yWindow="-6375" windowWidth="29610" windowHeight="15465" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Story" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="68">
   <si>
     <t>ScrollType</t>
   </si>
@@ -227,6 +227,9 @@
   <si>
     <t>TimelineTickInterval</t>
   </si>
+  <si>
+    <t>5y</t>
+  </si>
 </sst>
 </file>
 
@@ -330,7 +333,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -355,6 +358,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -581,29 +586,29 @@
     <col min="3" max="3" width="24.21875" customWidth="1"/>
     <col min="6" max="6" width="31.33203125" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
-    <col min="8" max="8" width="18.109375" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" customWidth="1"/>
     <col min="9" max="9" width="21.33203125" customWidth="1"/>
     <col min="10" max="10" width="17.44140625" customWidth="1"/>
     <col min="11" max="11" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
@@ -618,10 +623,10 @@
       <c r="J1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="6" t="s">
         <v>66</v>
       </c>
       <c r="M1" s="1"/>
@@ -660,14 +665,14 @@
       <c r="I2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="1">
-        <v>1950</v>
+      <c r="J2" s="12">
+        <v>1990</v>
       </c>
-      <c r="K2" s="1">
-        <v>1970</v>
+      <c r="K2" s="12">
+        <v>2030</v>
       </c>
-      <c r="L2" s="1">
-        <v>5</v>
+      <c r="L2" s="13" t="s">
+        <v>67</v>
       </c>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>

</xml_diff>